<commit_message>
fix: separate real-world legends from native-CR bars
</commit_message>
<xml_diff>
--- a/experiments/cr_native_no_btv_20260820/results/native_cr_no_btv_analysis_20260820.xlsx
+++ b/experiments/cr_native_no_btv_20260820/results/native_cr_no_btv_analysis_20260820.xlsx
@@ -536,7 +536,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="1809750"/>
+    <ext cx="7239000" cy="1727147"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -561,7 +561,7 @@
       <row>22</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="1809750"/>
+    <ext cx="7239000" cy="1727147"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>

</xml_diff>

<commit_message>
fix: restore legacy real-world legends
</commit_message>
<xml_diff>
--- a/experiments/cr_native_no_btv_20260820/results/native_cr_no_btv_analysis_20260820.xlsx
+++ b/experiments/cr_native_no_btv_20260820/results/native_cr_no_btv_analysis_20260820.xlsx
@@ -536,7 +536,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="1727147"/>
+    <ext cx="7239000" cy="1732153"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -561,7 +561,7 @@
       <row>22</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="1727147"/>
+    <ext cx="7239000" cy="1734656"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>

</xml_diff>